<commit_message>
Update the testcases and the CI/CD pipeline
</commit_message>
<xml_diff>
--- a/testData/searchProduct.xlsx
+++ b/testData/searchProduct.xlsx
@@ -371,7 +371,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -615,51 +615,204 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>Voltage</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>MixerModelY</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>500W</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>220V</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>MixerMoabccccccdelY</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>100500W</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>22440V</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>Voltage</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>MixerModelY</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>500W</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>220V</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>MixerMoabccccccdelY</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>100500W</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>22440V</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>Voltage</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>MixerModelY</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>500W</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>220V</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>MixerMoabccccccdelY</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>100500W</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>22440V</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Voltage</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MixerModelY</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>500W</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>220V</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MixerMoabccccccdelY</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>100500W</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
         <is>
           <t>22440V</t>
         </is>

</xml_diff>